<commit_message>
Add AOTA Report text file support and timing validation
Introduces a parser for AOTA_Report.txt files, enabling extraction of D/R times, uncertainties, and SNR for report generation. Updates the report dialog to support selection of both AOTA XML and AOTA Report files, with multi-event selection and cross-validation of timing data. Enhances help documentation and UI to reflect new workflow, and ensures that either AOTA XML or AOTA Report is required for Positive/Unsure observations. Adds logic to compare D/R times from both sources and warn if they differ by more than 0.1s.
</commit_message>
<xml_diff>
--- a/occultation-manager/python/RASNZ_AstReporttForm_V4.1.2.G_Template.xlsx
+++ b/occultation-manager/python/RASNZ_AstReporttForm_V4.1.2.G_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MichaelCamilleri\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="91" documentId="13_ncr:1_{8CDBA6B2-A7D7-42E4-8B26-C427C3DBEF8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C69CBF3-F058-4386-8661-69ACF2DCB3DE}"/>
+  <xr:revisionPtr revIDLastSave="94" documentId="13_ncr:1_{8CDBA6B2-A7D7-42E4-8B26-C427C3DBEF8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FECFF79-05B4-4F14-9E1F-CFC7CC244B43}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="2" xr2:uid="{080FCFD7-E308-408C-BE8B-98AE63D705D4}"/>
   </bookViews>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="504">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="505">
   <si>
     <t>Directions for Use of Asteroid Occultation Reporting Form</t>
   </si>
@@ -1342,7 +1342,7 @@
     <t>{{INTEGRATION_UNITS}}</t>
   </si>
   <si>
-    <t>{{OTHER_DETECTED_RELATED_INFO}}</t>
+    <t>{{OTHER_DETECTOR_RELATED_INFO}}</t>
   </si>
   <si>
     <t>Camera Delay Correction:</t>
@@ -1456,6 +1456,9 @@
     <t>{{STOPPED_OBSERVING_HOURS}}</t>
   </si>
   <si>
+    <t>{{STOPPED_OBSERVING_MINUTES}}</t>
+  </si>
+  <si>
     <t>{{STOPPED_OBSERVING_SECONDS}}</t>
   </si>
   <si>
@@ -1483,7 +1486,7 @@
     <t>S/N =</t>
   </si>
   <si>
-    <t>{SNR}</t>
+    <t>{{SNR}}</t>
   </si>
   <si>
     <t>(if known)</t>
@@ -9411,12 +9414,14 @@
       <c r="G37" s="20" t="s">
         <v>276</v>
       </c>
-      <c r="H37" s="93"/>
+      <c r="H37" s="93" t="s">
+        <v>393</v>
+      </c>
       <c r="I37" s="20" t="s">
         <v>276</v>
       </c>
       <c r="J37" s="204" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K37" s="204"/>
       <c r="L37" s="18"/>
@@ -9445,7 +9450,7 @@
       <c r="D38" s="115"/>
       <c r="E38" s="115"/>
       <c r="F38" s="12" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="G38" s="115"/>
       <c r="H38" s="7" t="s">
@@ -9453,7 +9458,7 @@
       </c>
       <c r="I38" s="7"/>
       <c r="J38" s="207" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="K38" s="196"/>
       <c r="L38" s="3"/>
@@ -9468,11 +9473,11 @@
       <c r="U38" s="115"/>
       <c r="V38" s="99"/>
       <c r="W38" s="208" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="X38" s="146"/>
       <c r="Y38" s="43" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="Z38" s="44"/>
       <c r="AA38" s="45"/>
@@ -9515,15 +9520,15 @@
       <c r="B40" s="126"/>
       <c r="C40" s="120"/>
       <c r="D40" s="106" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="E40" s="206" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="F40" s="206"/>
       <c r="G40" s="206"/>
       <c r="H40" s="18" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="I40" s="99"/>
       <c r="J40" s="99"/>
@@ -9538,15 +9543,15 @@
       <c r="S40" s="122"/>
       <c r="T40" s="122"/>
       <c r="U40" s="154" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="V40" s="155"/>
       <c r="W40" s="198" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="X40" s="198"/>
       <c r="Y40" s="196" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="Z40" s="197"/>
       <c r="AA40" s="197"/>
@@ -9559,7 +9564,7 @@
       <c r="C41" s="115"/>
       <c r="D41" s="115"/>
       <c r="E41" s="199" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F41" s="199"/>
       <c r="G41" s="122"/>
@@ -9588,12 +9593,12 @@
     </row>
     <row r="42" spans="1:29" ht="24" customHeight="1">
       <c r="A42" s="195" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B42" s="195"/>
       <c r="C42" s="195"/>
       <c r="D42" s="21" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="E42" s="22"/>
       <c r="F42" s="22"/>
@@ -9623,7 +9628,7 @@
     </row>
     <row r="43" spans="1:29" ht="24" customHeight="1">
       <c r="A43" s="195" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B43" s="195"/>
       <c r="C43" s="195"/>
@@ -9702,7 +9707,7 @@
       <c r="N45" s="126"/>
       <c r="O45" s="126"/>
       <c r="P45" s="126" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="Q45" s="126"/>
       <c r="R45" s="126"/>
@@ -9733,7 +9738,7 @@
       <c r="L46" s="99"/>
       <c r="M46" s="19"/>
       <c r="N46" s="19" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="O46" s="19"/>
       <c r="P46" s="19"/>
@@ -9790,7 +9795,7 @@
       <c r="B48" s="99"/>
       <c r="C48" s="99"/>
       <c r="D48" s="138" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E48" s="139"/>
       <c r="F48" s="139"/>
@@ -9989,7 +9994,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="24" customHeight="1">
       <c r="A1" s="139" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B1" s="213"/>
       <c r="C1" s="213"/>
@@ -10007,21 +10012,21 @@
     </row>
     <row r="4" spans="1:14" ht="15.95" customHeight="1">
       <c r="A4" s="213" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B4" s="213"/>
       <c r="C4" s="213"/>
       <c r="D4" s="213"/>
       <c r="E4" s="99"/>
       <c r="F4" s="213" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="G4" s="213"/>
       <c r="H4" s="213"/>
       <c r="I4" s="213"/>
       <c r="J4" s="99"/>
       <c r="K4" s="213" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="L4" s="213"/>
       <c r="M4" s="213"/>
@@ -10029,7 +10034,7 @@
     </row>
     <row r="5" spans="1:14" ht="15.95" customHeight="1">
       <c r="A5" s="213" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B5" s="179"/>
       <c r="C5" s="179"/>
@@ -10295,21 +10300,21 @@
     </row>
     <row r="19" spans="1:14" ht="15.95" customHeight="1">
       <c r="A19" s="213" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B19" s="213"/>
       <c r="C19" s="213"/>
       <c r="D19" s="213"/>
       <c r="E19" s="99"/>
       <c r="F19" s="213" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="G19" s="213"/>
       <c r="H19" s="213"/>
       <c r="I19" s="213"/>
       <c r="J19" s="99"/>
       <c r="K19" s="213" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="L19" s="213"/>
       <c r="M19" s="213"/>
@@ -10322,7 +10327,7 @@
       <c r="D20" s="99"/>
       <c r="E20" s="99"/>
       <c r="F20" s="216" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="G20" s="216"/>
       <c r="H20" s="216"/>
@@ -10344,7 +10349,7 @@
       <c r="D21" s="214"/>
       <c r="E21" s="99"/>
       <c r="F21" s="216" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="G21" s="216"/>
       <c r="H21" s="216"/>
@@ -10386,7 +10391,7 @@
       <c r="D23" s="214"/>
       <c r="E23" s="99"/>
       <c r="F23" s="217" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="G23" s="217"/>
       <c r="H23" s="217"/>
@@ -10428,7 +10433,7 @@
       <c r="D25" s="214"/>
       <c r="E25" s="99"/>
       <c r="F25" s="133" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="G25" s="133"/>
       <c r="H25" s="133"/>
@@ -10450,7 +10455,7 @@
       <c r="D26" s="214"/>
       <c r="E26" s="99"/>
       <c r="F26" s="133" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G26" s="133"/>
       <c r="H26" s="133"/>
@@ -10488,7 +10493,7 @@
       <c r="D28" s="214"/>
       <c r="E28" s="99"/>
       <c r="F28" s="133" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G28" s="133"/>
       <c r="H28" s="133"/>
@@ -10508,7 +10513,7 @@
       <c r="D29" s="214"/>
       <c r="E29" s="99"/>
       <c r="F29" s="133" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="G29" s="133"/>
       <c r="H29" s="133"/>
@@ -10546,7 +10551,7 @@
       <c r="D31" s="214"/>
       <c r="E31" s="99"/>
       <c r="F31" s="133" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="G31" s="133"/>
       <c r="H31" s="133"/>
@@ -10566,7 +10571,7 @@
       <c r="D32" s="214"/>
       <c r="E32" s="99"/>
       <c r="F32" s="133" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="G32" s="133"/>
       <c r="H32" s="133"/>
@@ -10599,7 +10604,7 @@
       <c r="D34" s="214"/>
       <c r="E34" s="99"/>
       <c r="F34" s="133" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="G34" s="133"/>
       <c r="H34" s="133"/>
@@ -10614,7 +10619,7 @@
       <c r="D35" s="214"/>
       <c r="E35" s="99"/>
       <c r="F35" s="133" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="G35" s="133"/>
       <c r="H35" s="133"/>
@@ -10642,7 +10647,7 @@
       <c r="D37" s="214"/>
       <c r="E37" s="99"/>
       <c r="F37" s="133" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="G37" s="133"/>
       <c r="H37" s="133"/>
@@ -10670,7 +10675,7 @@
       <c r="D39" s="214"/>
       <c r="E39" s="99"/>
       <c r="F39" s="133" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="G39" s="133"/>
       <c r="H39" s="133"/>
@@ -10698,7 +10703,7 @@
       <c r="D41" s="214"/>
       <c r="E41" s="99"/>
       <c r="F41" s="217" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="G41" s="217"/>
       <c r="H41" s="217"/>
@@ -10954,7 +10959,7 @@
   <sheetData>
     <row r="2" spans="1:16" ht="21.75" customHeight="1">
       <c r="A2" s="139" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B2" s="181"/>
       <c r="C2" s="181"/>
@@ -10975,7 +10980,7 @@
     <row r="5" spans="1:16" ht="26.1" customHeight="1">
       <c r="A5" s="99"/>
       <c r="B5" s="224" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C5" s="221"/>
       <c r="D5" s="221"/>
@@ -10995,14 +11000,14 @@
     <row r="6" spans="1:16" ht="18" customHeight="1">
       <c r="A6" s="99"/>
       <c r="B6" s="218" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C6" s="179"/>
       <c r="D6" s="179" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E6" s="179" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F6" s="219"/>
       <c r="G6" s="179"/>
@@ -11010,7 +11015,7 @@
       <c r="I6" s="99"/>
       <c r="J6" s="99"/>
       <c r="K6" s="139" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="L6" s="139"/>
       <c r="M6" s="139"/>
@@ -11021,17 +11026,17 @@
     <row r="7" spans="1:16" ht="18" customHeight="1">
       <c r="A7" s="99"/>
       <c r="B7" s="136" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C7" s="115" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D7" s="179"/>
       <c r="E7" s="115" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F7" s="134" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G7" s="115"/>
       <c r="H7" s="115"/>
@@ -11047,10 +11052,10 @@
     <row r="8" spans="1:16" ht="14.1" customHeight="1">
       <c r="A8" s="99"/>
       <c r="B8" s="136" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C8" s="115" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D8" s="115">
         <v>2</v>
@@ -11066,12 +11071,12 @@
       <c r="I8" s="99"/>
       <c r="J8" s="99"/>
       <c r="K8" s="220" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="L8" s="220"/>
       <c r="M8" s="220"/>
       <c r="N8" s="228" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="O8" s="228"/>
       <c r="P8" s="115"/>
@@ -11079,10 +11084,10 @@
     <row r="9" spans="1:16" ht="14.1" customHeight="1">
       <c r="A9" s="99"/>
       <c r="B9" s="136" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C9" s="115" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D9" s="115">
         <v>3</v>
@@ -11098,7 +11103,7 @@
       <c r="I9" s="99"/>
       <c r="J9" s="99"/>
       <c r="K9" s="220" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="L9" s="220"/>
       <c r="M9" s="220"/>
@@ -11111,10 +11116,10 @@
     <row r="10" spans="1:16" ht="14.1" customHeight="1">
       <c r="A10" s="99"/>
       <c r="B10" s="136" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C10" s="115" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D10" s="115">
         <v>5</v>
@@ -11130,12 +11135,12 @@
       <c r="I10" s="99"/>
       <c r="J10" s="99"/>
       <c r="K10" s="220" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="L10" s="220"/>
       <c r="M10" s="220"/>
       <c r="N10" s="228" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="O10" s="228"/>
       <c r="P10" s="115"/>
@@ -11143,10 +11148,10 @@
     <row r="11" spans="1:16" ht="14.1" customHeight="1">
       <c r="A11" s="99"/>
       <c r="B11" s="136" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C11" s="115" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D11" s="115">
         <v>9</v>
@@ -11162,7 +11167,7 @@
       <c r="I11" s="99"/>
       <c r="J11" s="99"/>
       <c r="K11" s="220" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="L11" s="220"/>
       <c r="M11" s="220"/>
@@ -11175,10 +11180,10 @@
     <row r="12" spans="1:16" ht="14.1" customHeight="1">
       <c r="A12" s="99"/>
       <c r="B12" s="136" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C12" s="115" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D12" s="115">
         <v>17</v>
@@ -11203,10 +11208,10 @@
     <row r="13" spans="1:16" ht="14.1" customHeight="1">
       <c r="A13" s="99"/>
       <c r="B13" s="136" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C13" s="115" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D13" s="115">
         <v>33</v>
@@ -11231,10 +11236,10 @@
     <row r="14" spans="1:16" ht="14.1" customHeight="1">
       <c r="A14" s="99"/>
       <c r="B14" s="136" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C14" s="115" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D14" s="115">
         <v>65</v>
@@ -11259,10 +11264,10 @@
     <row r="15" spans="1:16" ht="14.1" customHeight="1">
       <c r="A15" s="99"/>
       <c r="B15" s="136" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C15" s="115" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D15" s="115">
         <v>129</v>
@@ -11287,10 +11292,10 @@
     <row r="16" spans="1:16" ht="14.1" customHeight="1">
       <c r="A16" s="99"/>
       <c r="B16" s="136" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C16" s="115" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D16" s="115">
         <v>257</v>
@@ -11314,10 +11319,10 @@
     </row>
     <row r="17" spans="2:16" ht="14.1" customHeight="1">
       <c r="B17" s="75" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C17" s="76" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="D17" s="76">
         <v>513</v>
@@ -11341,7 +11346,7 @@
     </row>
     <row r="20" spans="2:16" ht="26.1" customHeight="1">
       <c r="B20" s="224" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C20" s="221"/>
       <c r="D20" s="221"/>
@@ -11360,21 +11365,21 @@
     </row>
     <row r="21" spans="2:16" ht="18" customHeight="1">
       <c r="B21" s="218" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C21" s="179"/>
       <c r="D21" s="179" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E21" s="179" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F21" s="219"/>
       <c r="G21" s="179"/>
       <c r="H21" s="179"/>
       <c r="I21" s="99"/>
       <c r="J21" s="139" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K21" s="179"/>
       <c r="L21" s="179"/>
@@ -11385,39 +11390,39 @@
     </row>
     <row r="22" spans="2:16" ht="18" customHeight="1">
       <c r="B22" s="136" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C22" s="115" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D22" s="179"/>
       <c r="E22" s="115" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F22" s="134" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G22" s="115"/>
       <c r="H22" s="115"/>
       <c r="I22" s="99"/>
       <c r="J22" s="179" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="K22" s="181"/>
       <c r="L22" s="181"/>
       <c r="M22" s="99"/>
       <c r="N22" s="179" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="O22" s="179"/>
       <c r="P22" s="181"/>
     </row>
     <row r="23" spans="2:16" ht="14.1" customHeight="1">
       <c r="B23" s="136" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C23" s="115" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="D23" s="115">
         <v>1</v>
@@ -11432,23 +11437,23 @@
       <c r="H23" s="99"/>
       <c r="I23" s="99"/>
       <c r="J23" s="179" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="K23" s="181"/>
       <c r="L23" s="181"/>
       <c r="M23" s="99"/>
       <c r="N23" s="179" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="O23" s="179"/>
       <c r="P23" s="181"/>
     </row>
     <row r="24" spans="2:16" ht="14.1" customHeight="1">
       <c r="B24" s="136" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C24" s="115" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="D24" s="115">
         <v>2</v>
@@ -11465,23 +11470,23 @@
       <c r="H24" s="99"/>
       <c r="I24" s="99"/>
       <c r="J24" s="179" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K24" s="181"/>
       <c r="L24" s="181"/>
       <c r="M24" s="99"/>
       <c r="N24" s="179" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="O24" s="179"/>
       <c r="P24" s="181"/>
     </row>
     <row r="25" spans="2:16" ht="14.1" customHeight="1">
       <c r="B25" s="136" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C25" s="115" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="D25" s="115">
         <v>4</v>
@@ -11497,7 +11502,7 @@
       <c r="H25" s="99"/>
       <c r="I25" s="99"/>
       <c r="J25" s="179" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="K25" s="179"/>
       <c r="L25" s="179"/>
@@ -11508,10 +11513,10 @@
     </row>
     <row r="26" spans="2:16" ht="14.1" customHeight="1">
       <c r="B26" s="136" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C26" s="115" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D26" s="115">
         <v>8</v>
@@ -11536,10 +11541,10 @@
     </row>
     <row r="27" spans="2:16" ht="14.1" customHeight="1">
       <c r="B27" s="136" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C27" s="115" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="D27" s="115">
         <v>16</v>
@@ -11564,10 +11569,10 @@
     </row>
     <row r="28" spans="2:16" ht="14.1" customHeight="1">
       <c r="B28" s="136" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C28" s="115" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D28" s="115">
         <v>32</v>
@@ -11592,10 +11597,10 @@
     </row>
     <row r="29" spans="2:16" ht="14.1" customHeight="1">
       <c r="B29" s="136" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C29" s="115" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="D29" s="115">
         <v>64</v>
@@ -11620,10 +11625,10 @@
     </row>
     <row r="30" spans="2:16" ht="14.1" customHeight="1">
       <c r="B30" s="136" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C30" s="115" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="D30" s="115">
         <v>128</v>
@@ -11648,10 +11653,10 @@
     </row>
     <row r="31" spans="2:16" ht="14.1" customHeight="1">
       <c r="B31" s="75" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C31" s="76" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="D31" s="76">
         <v>256</v>
@@ -11701,7 +11706,7 @@
     </row>
     <row r="34" spans="2:8" ht="26.1" customHeight="1">
       <c r="B34" s="224" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C34" s="221"/>
       <c r="D34" s="221"/>
@@ -11712,14 +11717,14 @@
     </row>
     <row r="35" spans="2:8" ht="18" customHeight="1">
       <c r="B35" s="218" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C35" s="179"/>
       <c r="D35" s="179" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E35" s="179" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F35" s="219"/>
       <c r="G35" s="179"/>
@@ -11727,22 +11732,22 @@
     </row>
     <row r="36" spans="2:8" ht="18" customHeight="1">
       <c r="B36" s="136" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C36" s="115"/>
       <c r="D36" s="179"/>
       <c r="E36" s="115" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F36" s="134" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G36" s="115"/>
       <c r="H36" s="115"/>
     </row>
     <row r="37" spans="2:8" ht="14.1" customHeight="1">
       <c r="B37" s="136" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C37" s="115"/>
       <c r="D37" s="115">
@@ -11757,7 +11762,7 @@
     </row>
     <row r="38" spans="2:8" ht="14.1" customHeight="1">
       <c r="B38" s="136" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C38" s="115"/>
       <c r="D38" s="115">
@@ -11773,7 +11778,7 @@
     </row>
     <row r="39" spans="2:8" ht="14.1" customHeight="1">
       <c r="B39" s="136" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C39" s="115"/>
       <c r="D39" s="115">
@@ -11788,7 +11793,7 @@
     </row>
     <row r="40" spans="2:8" ht="14.1" customHeight="1">
       <c r="B40" s="136" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C40" s="115"/>
       <c r="D40" s="115">
@@ -11803,7 +11808,7 @@
     </row>
     <row r="41" spans="2:8" ht="14.1" customHeight="1">
       <c r="B41" s="136" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C41" s="115"/>
       <c r="D41" s="115">
@@ -11818,7 +11823,7 @@
     </row>
     <row r="42" spans="2:8" ht="14.1" customHeight="1">
       <c r="B42" s="136" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C42" s="115"/>
       <c r="D42" s="115">
@@ -11833,7 +11838,7 @@
     </row>
     <row r="43" spans="2:8" ht="14.1" customHeight="1">
       <c r="B43" s="136" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C43" s="115"/>
       <c r="D43" s="115">
@@ -11848,7 +11853,7 @@
     </row>
     <row r="44" spans="2:8" ht="14.1" customHeight="1">
       <c r="B44" s="136" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C44" s="115"/>
       <c r="D44" s="115">
@@ -11863,7 +11868,7 @@
     </row>
     <row r="45" spans="2:8" ht="14.1" customHeight="1">
       <c r="B45" s="75" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C45" s="76"/>
       <c r="D45" s="76">
@@ -11878,7 +11883,7 @@
     </row>
     <row r="48" spans="2:8" ht="26.1" customHeight="1">
       <c r="B48" s="221" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="C48" s="221"/>
       <c r="D48" s="221"/>
@@ -11889,14 +11894,14 @@
     </row>
     <row r="49" spans="2:8" ht="18" customHeight="1">
       <c r="B49" s="179" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C49" s="179"/>
       <c r="D49" s="179" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E49" s="179" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F49" s="219"/>
       <c r="G49" s="179"/>
@@ -11907,17 +11912,17 @@
       <c r="C50" s="99"/>
       <c r="D50" s="179"/>
       <c r="E50" s="115" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F50" s="134" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G50" s="115"/>
       <c r="H50" s="115"/>
     </row>
     <row r="51" spans="2:8" ht="14.1" customHeight="1">
       <c r="B51" s="115" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C51" s="99"/>
       <c r="D51" s="115">
@@ -11934,7 +11939,7 @@
     </row>
     <row r="52" spans="2:8" ht="14.1" customHeight="1">
       <c r="B52" s="115" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C52" s="99"/>
       <c r="D52" s="115">
@@ -11951,7 +11956,7 @@
     </row>
     <row r="53" spans="2:8" ht="14.1" customHeight="1">
       <c r="B53" s="115" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C53" s="99"/>
       <c r="D53" s="115">
@@ -11968,7 +11973,7 @@
     </row>
     <row r="54" spans="2:8" ht="14.1" customHeight="1">
       <c r="B54" s="107" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C54" s="79"/>
       <c r="D54" s="107">
@@ -11985,7 +11990,7 @@
     </row>
     <row r="55" spans="2:8" ht="14.1" customHeight="1">
       <c r="B55" s="115" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C55" s="99"/>
       <c r="D55" s="115">
@@ -12002,7 +12007,7 @@
     </row>
     <row r="56" spans="2:8" ht="14.1" customHeight="1">
       <c r="B56" s="107" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="C56" s="79"/>
       <c r="D56" s="107">
@@ -12019,7 +12024,7 @@
     </row>
     <row r="57" spans="2:8" ht="14.1" customHeight="1">
       <c r="B57" s="107" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C57" s="79"/>
       <c r="D57" s="107">
@@ -12036,7 +12041,7 @@
     </row>
     <row r="58" spans="2:8" ht="14.1" customHeight="1">
       <c r="B58" s="107" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C58" s="79"/>
       <c r="D58" s="107">
@@ -12053,7 +12058,7 @@
     </row>
     <row r="59" spans="2:8" ht="14.1" customHeight="1">
       <c r="B59" s="115" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C59" s="99"/>
       <c r="D59" s="115">
@@ -12070,7 +12075,7 @@
     </row>
     <row r="60" spans="2:8" ht="14.1" customHeight="1">
       <c r="B60" s="107" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="C60" s="79"/>
       <c r="D60" s="107">
@@ -12087,7 +12092,7 @@
     </row>
     <row r="61" spans="2:8" ht="14.1" customHeight="1">
       <c r="B61" s="115" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C61" s="99"/>
       <c r="D61" s="119">
@@ -12104,7 +12109,7 @@
     </row>
     <row r="62" spans="2:8" ht="14.1" customHeight="1">
       <c r="B62" s="107" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="C62" s="79"/>
       <c r="D62" s="107">
@@ -12121,7 +12126,7 @@
     </row>
     <row r="63" spans="2:8" ht="14.1" customHeight="1">
       <c r="B63" s="76" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C63" s="80"/>
       <c r="D63" s="76">
@@ -12138,7 +12143,7 @@
     </row>
     <row r="64" spans="2:8" ht="14.1" customHeight="1">
       <c r="B64" s="223" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="C64" s="223"/>
       <c r="D64" s="223"/>
@@ -12149,7 +12154,7 @@
     </row>
     <row r="67" spans="2:8" ht="26.1" customHeight="1">
       <c r="B67" s="224" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="C67" s="221"/>
       <c r="D67" s="221"/>
@@ -12160,14 +12165,14 @@
     </row>
     <row r="68" spans="2:8" ht="18" customHeight="1">
       <c r="B68" s="218" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C68" s="179"/>
       <c r="D68" s="179" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E68" s="179" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F68" s="219"/>
       <c r="G68" s="179"/>
@@ -12175,22 +12180,22 @@
     </row>
     <row r="69" spans="2:8" ht="18" customHeight="1">
       <c r="B69" s="136" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="C69" s="99"/>
       <c r="D69" s="179"/>
       <c r="E69" s="115" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F69" s="134" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G69" s="115"/>
       <c r="H69" s="115"/>
     </row>
     <row r="70" spans="2:8" ht="14.1" customHeight="1">
       <c r="B70" s="136" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C70" s="99"/>
       <c r="D70" s="115">
@@ -12207,7 +12212,7 @@
     </row>
     <row r="71" spans="2:8" ht="14.1" customHeight="1">
       <c r="B71" s="136" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="C71" s="99"/>
       <c r="D71" s="115">
@@ -12224,7 +12229,7 @@
     </row>
     <row r="72" spans="2:8" ht="14.1" customHeight="1">
       <c r="B72" s="136" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C72" s="99"/>
       <c r="D72" s="115">
@@ -12241,7 +12246,7 @@
     </row>
     <row r="73" spans="2:8" ht="14.1" customHeight="1">
       <c r="B73" s="110" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="C73" s="111"/>
       <c r="D73" s="107">
@@ -12258,7 +12263,7 @@
     </row>
     <row r="74" spans="2:8" ht="14.1" customHeight="1">
       <c r="B74" s="136" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C74" s="99"/>
       <c r="D74" s="115">
@@ -12275,7 +12280,7 @@
     </row>
     <row r="75" spans="2:8" ht="14.1" customHeight="1">
       <c r="B75" s="110" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="C75" s="111"/>
       <c r="D75" s="107">
@@ -12292,7 +12297,7 @@
     </row>
     <row r="76" spans="2:8" ht="14.1" customHeight="1">
       <c r="B76" s="136" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="C76" s="99"/>
       <c r="D76" s="115">
@@ -12309,7 +12314,7 @@
     </row>
     <row r="77" spans="2:8" ht="14.1" customHeight="1">
       <c r="B77" s="110" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="C77" s="111"/>
       <c r="D77" s="107">
@@ -12326,7 +12331,7 @@
     </row>
     <row r="78" spans="2:8" ht="14.1" customHeight="1">
       <c r="B78" s="136" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="C78" s="99"/>
       <c r="D78" s="115">
@@ -12343,7 +12348,7 @@
     </row>
     <row r="79" spans="2:8" ht="14.1" customHeight="1">
       <c r="B79" s="110" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="C79" s="111"/>
       <c r="D79" s="107">
@@ -12360,7 +12365,7 @@
     </row>
     <row r="80" spans="2:8" ht="14.1" customHeight="1">
       <c r="B80" s="136" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="C80" s="99"/>
       <c r="D80" s="115">
@@ -12377,7 +12382,7 @@
     </row>
     <row r="81" spans="2:8" ht="14.1" customHeight="1">
       <c r="B81" s="110" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="C81" s="111"/>
       <c r="D81" s="107">
@@ -12394,7 +12399,7 @@
     </row>
     <row r="82" spans="2:8" ht="14.1" customHeight="1">
       <c r="B82" s="75" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C82" s="80"/>
       <c r="D82" s="76">
@@ -12411,7 +12416,7 @@
     </row>
     <row r="83" spans="2:8" ht="14.1" customHeight="1">
       <c r="B83" s="223" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="C83" s="223"/>
       <c r="D83" s="223"/>
@@ -12422,7 +12427,7 @@
     </row>
     <row r="86" spans="2:8" ht="26.1" customHeight="1">
       <c r="B86" s="225" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C86" s="226"/>
       <c r="D86" s="226"/>
@@ -12433,14 +12438,14 @@
     </row>
     <row r="87" spans="2:8" ht="18" customHeight="1">
       <c r="B87" s="218" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C87" s="179"/>
       <c r="D87" s="179" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E87" s="179" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F87" s="219"/>
       <c r="G87" s="179"/>
@@ -12451,17 +12456,17 @@
       <c r="C88" s="99"/>
       <c r="D88" s="179"/>
       <c r="E88" s="115" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F88" s="134" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G88" s="115"/>
       <c r="H88" s="115"/>
     </row>
     <row r="89" spans="2:8" ht="14.1" customHeight="1">
       <c r="B89" s="136" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C89" s="115"/>
       <c r="D89" s="115">
@@ -12476,7 +12481,7 @@
     </row>
     <row r="90" spans="2:8" ht="14.1" customHeight="1">
       <c r="B90" s="136" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C90" s="115"/>
       <c r="D90" s="115">
@@ -12491,7 +12496,7 @@
     </row>
     <row r="91" spans="2:8" ht="14.1" customHeight="1">
       <c r="B91" s="136" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C91" s="115"/>
       <c r="D91" s="115">
@@ -12506,7 +12511,7 @@
     </row>
     <row r="92" spans="2:8" ht="14.1" customHeight="1">
       <c r="B92" s="136" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C92" s="115"/>
       <c r="D92" s="115">
@@ -12521,7 +12526,7 @@
     </row>
     <row r="93" spans="2:8" ht="14.1" customHeight="1">
       <c r="B93" s="136" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C93" s="115"/>
       <c r="D93" s="115">
@@ -12536,7 +12541,7 @@
     </row>
     <row r="94" spans="2:8" ht="14.1" customHeight="1">
       <c r="B94" s="136" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="C94" s="115"/>
       <c r="D94" s="115">
@@ -12551,7 +12556,7 @@
     </row>
     <row r="95" spans="2:8" ht="14.1" customHeight="1">
       <c r="B95" s="136" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="C95" s="115"/>
       <c r="D95" s="115">
@@ -12566,7 +12571,7 @@
     </row>
     <row r="96" spans="2:8" ht="14.1" customHeight="1">
       <c r="B96" s="136" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C96" s="115"/>
       <c r="D96" s="115">
@@ -12581,7 +12586,7 @@
     </row>
     <row r="97" spans="2:6" ht="14.1" customHeight="1">
       <c r="B97" s="136" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C97" s="115"/>
       <c r="D97" s="115">
@@ -12594,7 +12599,7 @@
     </row>
     <row r="98" spans="2:6" ht="14.1" customHeight="1">
       <c r="B98" s="136" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C98" s="115"/>
       <c r="D98" s="115">
@@ -12607,7 +12612,7 @@
     </row>
     <row r="99" spans="2:6" ht="14.1" customHeight="1">
       <c r="B99" s="136" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C99" s="115"/>
       <c r="D99" s="115">
@@ -12620,7 +12625,7 @@
     </row>
     <row r="100" spans="2:6" ht="14.1" customHeight="1">
       <c r="B100" s="136" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C100" s="115"/>
       <c r="D100" s="115">
@@ -12633,7 +12638,7 @@
     </row>
     <row r="101" spans="2:6" ht="14.1" customHeight="1">
       <c r="B101" s="136" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C101" s="115"/>
       <c r="D101" s="115">
@@ -12646,7 +12651,7 @@
     </row>
     <row r="102" spans="2:6" ht="14.1" customHeight="1">
       <c r="B102" s="136" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C102" s="115"/>
       <c r="D102" s="115">
@@ -12659,7 +12664,7 @@
     </row>
     <row r="103" spans="2:6" ht="14.1" customHeight="1">
       <c r="B103" s="75" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C103" s="76"/>
       <c r="D103" s="76">

</xml_diff>

<commit_message>
Added OTE to report
</commit_message>
<xml_diff>
--- a/occultation-manager/python/RASNZ_AstReporttForm_V4.1.2.G_Template.xlsx
+++ b/occultation-manager/python/RASNZ_AstReporttForm_V4.1.2.G_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29622"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29704"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MichaelCamilleri\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="94" documentId="13_ncr:1_{8CDBA6B2-A7D7-42E4-8B26-C427C3DBEF8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FECFF79-05B4-4F14-9E1F-CFC7CC244B43}"/>
+  <xr:revisionPtr revIDLastSave="95" documentId="13_ncr:1_{8CDBA6B2-A7D7-42E4-8B26-C427C3DBEF8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB57929E-64DA-4421-BFB4-EC47FC9C0F7C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="2" xr2:uid="{080FCFD7-E308-408C-BE8B-98AE63D705D4}"/>
   </bookViews>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="506">
   <si>
     <t>Directions for Use of Asteroid Occultation Reporting Form</t>
   </si>
@@ -1301,6 +1301,9 @@
   </si>
   <si>
     <t>OTA Used:</t>
+  </si>
+  <si>
+    <t>{{OTE}}</t>
   </si>
   <si>
     <t>Some of the cells in row 25 are  free form.  Look at Comments provided.</t>
@@ -7123,7 +7126,7 @@
       <c r="B27" s="99"/>
       <c r="C27" s="99">
         <f ca="1">YEAR(NOW())-1</f>
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D27" s="99"/>
       <c r="E27" s="99"/>
@@ -7138,7 +7141,7 @@
       <c r="B28" s="99"/>
       <c r="C28" s="99">
         <f ca="1">C27+1</f>
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D28" s="99"/>
       <c r="E28" s="99"/>
@@ -7155,7 +7158,7 @@
       <c r="B29" s="99"/>
       <c r="C29" s="99">
         <f ca="1">C28+1</f>
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="D29" s="99"/>
       <c r="E29" s="99"/>
@@ -7172,7 +7175,7 @@
       <c r="B30" s="99"/>
       <c r="C30" s="99">
         <f ca="1">C29+1</f>
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="D30" s="99"/>
       <c r="E30" s="99"/>
@@ -7187,7 +7190,7 @@
       <c r="B31" s="99"/>
       <c r="C31" s="99">
         <f ca="1">C30+1</f>
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="D31" s="99"/>
       <c r="E31" s="99"/>
@@ -7202,7 +7205,7 @@
       <c r="B32" s="99"/>
       <c r="C32" s="99">
         <f ca="1">C31+1</f>
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="D32" s="99"/>
       <c r="E32" s="99"/>
@@ -8844,7 +8847,9 @@
       </c>
       <c r="M23" s="155"/>
       <c r="N23" s="155"/>
-      <c r="O23" s="163"/>
+      <c r="O23" s="163" t="s">
+        <v>342</v>
+      </c>
       <c r="P23" s="164"/>
       <c r="Q23" s="164"/>
       <c r="R23" s="164"/>
@@ -8866,7 +8871,7 @@
     </row>
     <row r="24" spans="1:30" ht="15.95" customHeight="1">
       <c r="A24" s="191" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B24" s="191"/>
       <c r="C24" s="191"/>
@@ -8878,13 +8883,13 @@
       <c r="I24" s="191"/>
       <c r="J24" s="191"/>
       <c r="K24" s="35" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="L24" s="115"/>
       <c r="M24" s="115"/>
       <c r="N24" s="99"/>
       <c r="O24" s="27" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="P24" s="99"/>
       <c r="Q24" s="99"/>
@@ -8893,7 +8898,7 @@
       <c r="T24" s="99"/>
       <c r="U24" s="99"/>
       <c r="V24" s="57" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="W24" s="99"/>
       <c r="X24" s="99"/>
@@ -8906,15 +8911,15 @@
     </row>
     <row r="25" spans="1:30" ht="15.95" customHeight="1">
       <c r="A25" s="141" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B25" s="141"/>
       <c r="C25" s="99" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D25" s="99"/>
       <c r="E25" s="193" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F25" s="193"/>
       <c r="G25" s="193"/>
@@ -8922,30 +8927,30 @@
       <c r="I25" s="193"/>
       <c r="J25" s="115"/>
       <c r="K25" s="27" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L25" s="192" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="M25" s="192"/>
       <c r="N25" s="142" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="O25" s="142"/>
       <c r="P25" s="89" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="Q25" s="99"/>
       <c r="R25" s="27" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="S25" s="171" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="T25" s="171"/>
       <c r="U25" s="27"/>
       <c r="V25" s="187" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="W25" s="187"/>
       <c r="X25" s="187"/>
@@ -8968,48 +8973,48 @@
       <c r="I26" s="116"/>
       <c r="J26" s="116"/>
       <c r="K26" s="165" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="L26" s="165"/>
       <c r="M26" s="165"/>
       <c r="N26" s="165"/>
       <c r="O26" s="165"/>
       <c r="P26" s="83" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="Q26" s="182" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="R26" s="183"/>
       <c r="S26" s="183"/>
       <c r="T26" s="183"/>
       <c r="U26" s="183"/>
       <c r="V26" s="85" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="W26" s="99" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="X26" s="99" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="Y26" s="99"/>
       <c r="Z26" s="99"/>
       <c r="AA26" s="99"/>
       <c r="AB26" s="27"/>
       <c r="AC26" s="84" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="AD26" s="99"/>
     </row>
     <row r="27" spans="1:30" ht="15.95" customHeight="1">
       <c r="A27" s="139" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B27" s="139"/>
       <c r="C27" s="126"/>
       <c r="D27" s="142" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E27" s="142"/>
       <c r="F27" s="142"/>
@@ -9022,7 +9027,7 @@
       <c r="K27" s="158"/>
       <c r="L27" s="126"/>
       <c r="M27" s="142" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="N27" s="142"/>
       <c r="O27" s="142"/>
@@ -9032,7 +9037,7 @@
       <c r="S27" s="158"/>
       <c r="T27" s="126"/>
       <c r="U27" s="166" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="V27" s="166"/>
       <c r="W27" s="166"/>
@@ -9078,12 +9083,12 @@
     </row>
     <row r="29" spans="1:30" ht="15.95" customHeight="1">
       <c r="A29" s="141" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B29" s="141"/>
       <c r="C29" s="141"/>
       <c r="D29" s="185" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E29" s="186"/>
       <c r="F29" s="186"/>
@@ -9119,7 +9124,7 @@
       <c r="D30" s="115"/>
       <c r="E30" s="115"/>
       <c r="F30" s="179" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="G30" s="179"/>
       <c r="H30" s="179"/>
@@ -9128,21 +9133,21 @@
       <c r="K30" s="179"/>
       <c r="L30" s="115"/>
       <c r="M30" s="170" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="N30" s="170"/>
       <c r="O30" s="119" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="P30" s="170" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="Q30" s="179"/>
       <c r="R30" s="179"/>
       <c r="S30" s="179"/>
       <c r="T30" s="179"/>
       <c r="U30" s="211" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="V30" s="211"/>
       <c r="W30" s="211"/>
@@ -9156,26 +9161,26 @@
     </row>
     <row r="31" spans="1:30" ht="15.95" customHeight="1">
       <c r="A31" s="142" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B31" s="142"/>
       <c r="C31" s="142"/>
       <c r="D31" s="142"/>
       <c r="E31" s="142"/>
       <c r="F31" s="90" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="G31" s="20" t="s">
         <v>276</v>
       </c>
       <c r="H31" s="91" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="I31" s="20" t="s">
         <v>276</v>
       </c>
       <c r="J31" s="212" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="K31" s="212"/>
       <c r="L31" s="18"/>
@@ -9200,7 +9205,7 @@
     </row>
     <row r="32" spans="1:30" ht="15.95" customHeight="1">
       <c r="A32" s="142" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B32" s="159"/>
       <c r="C32" s="159"/>
@@ -9238,31 +9243,31 @@
     </row>
     <row r="33" spans="1:29" ht="15.95" customHeight="1">
       <c r="A33" s="154" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B33" s="159"/>
       <c r="C33" s="159"/>
       <c r="D33" s="159"/>
       <c r="E33" s="159"/>
       <c r="F33" s="94" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="G33" s="20" t="s">
         <v>276</v>
       </c>
       <c r="H33" s="95" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="I33" s="20" t="s">
         <v>276</v>
       </c>
       <c r="J33" s="174" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="K33" s="174"/>
       <c r="L33" s="18"/>
       <c r="M33" s="200" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="N33" s="200"/>
       <c r="O33" s="98"/>
@@ -9283,7 +9288,7 @@
     </row>
     <row r="34" spans="1:29" ht="15.95" customHeight="1">
       <c r="A34" s="142" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B34" s="159"/>
       <c r="C34" s="159"/>
@@ -9320,31 +9325,31 @@
     </row>
     <row r="35" spans="1:29" ht="15.95" customHeight="1">
       <c r="A35" s="154" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B35" s="159"/>
       <c r="C35" s="159"/>
       <c r="D35" s="159"/>
       <c r="E35" s="159"/>
       <c r="F35" s="96" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G35" s="20" t="s">
         <v>276</v>
       </c>
       <c r="H35" s="97" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="I35" s="20" t="s">
         <v>276</v>
       </c>
       <c r="J35" s="194" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K35" s="194"/>
       <c r="L35" s="18"/>
       <c r="M35" s="205" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="N35" s="205"/>
       <c r="O35" s="98"/>
@@ -9365,7 +9370,7 @@
     </row>
     <row r="36" spans="1:29" ht="15.95" customHeight="1">
       <c r="A36" s="142" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B36" s="159"/>
       <c r="C36" s="159"/>
@@ -9402,26 +9407,26 @@
     </row>
     <row r="37" spans="1:29" ht="15.95" customHeight="1">
       <c r="A37" s="142" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B37" s="159"/>
       <c r="C37" s="159"/>
       <c r="D37" s="159"/>
       <c r="E37" s="159"/>
       <c r="F37" s="92" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="G37" s="20" t="s">
         <v>276</v>
       </c>
       <c r="H37" s="93" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="I37" s="20" t="s">
         <v>276</v>
       </c>
       <c r="J37" s="204" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="K37" s="204"/>
       <c r="L37" s="18"/>
@@ -9450,7 +9455,7 @@
       <c r="D38" s="115"/>
       <c r="E38" s="115"/>
       <c r="F38" s="12" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="G38" s="115"/>
       <c r="H38" s="7" t="s">
@@ -9458,7 +9463,7 @@
       </c>
       <c r="I38" s="7"/>
       <c r="J38" s="207" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="K38" s="196"/>
       <c r="L38" s="3"/>
@@ -9473,11 +9478,11 @@
       <c r="U38" s="115"/>
       <c r="V38" s="99"/>
       <c r="W38" s="208" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="X38" s="146"/>
       <c r="Y38" s="43" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="Z38" s="44"/>
       <c r="AA38" s="45"/>
@@ -9520,15 +9525,15 @@
       <c r="B40" s="126"/>
       <c r="C40" s="120"/>
       <c r="D40" s="106" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E40" s="206" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F40" s="206"/>
       <c r="G40" s="206"/>
       <c r="H40" s="18" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="I40" s="99"/>
       <c r="J40" s="99"/>
@@ -9543,15 +9548,15 @@
       <c r="S40" s="122"/>
       <c r="T40" s="122"/>
       <c r="U40" s="154" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="V40" s="155"/>
       <c r="W40" s="198" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="X40" s="198"/>
       <c r="Y40" s="196" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="Z40" s="197"/>
       <c r="AA40" s="197"/>
@@ -9564,7 +9569,7 @@
       <c r="C41" s="115"/>
       <c r="D41" s="115"/>
       <c r="E41" s="199" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F41" s="199"/>
       <c r="G41" s="122"/>
@@ -9593,12 +9598,12 @@
     </row>
     <row r="42" spans="1:29" ht="24" customHeight="1">
       <c r="A42" s="195" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B42" s="195"/>
       <c r="C42" s="195"/>
       <c r="D42" s="21" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="E42" s="22"/>
       <c r="F42" s="22"/>
@@ -9628,7 +9633,7 @@
     </row>
     <row r="43" spans="1:29" ht="24" customHeight="1">
       <c r="A43" s="195" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B43" s="195"/>
       <c r="C43" s="195"/>
@@ -9707,7 +9712,7 @@
       <c r="N45" s="126"/>
       <c r="O45" s="126"/>
       <c r="P45" s="126" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="Q45" s="126"/>
       <c r="R45" s="126"/>
@@ -9738,7 +9743,7 @@
       <c r="L46" s="99"/>
       <c r="M46" s="19"/>
       <c r="N46" s="19" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="O46" s="19"/>
       <c r="P46" s="19"/>
@@ -9795,7 +9800,7 @@
       <c r="B48" s="99"/>
       <c r="C48" s="99"/>
       <c r="D48" s="138" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="E48" s="139"/>
       <c r="F48" s="139"/>
@@ -9994,7 +9999,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="24" customHeight="1">
       <c r="A1" s="139" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B1" s="213"/>
       <c r="C1" s="213"/>
@@ -10012,21 +10017,21 @@
     </row>
     <row r="4" spans="1:14" ht="15.95" customHeight="1">
       <c r="A4" s="213" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B4" s="213"/>
       <c r="C4" s="213"/>
       <c r="D4" s="213"/>
       <c r="E4" s="99"/>
       <c r="F4" s="213" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="G4" s="213"/>
       <c r="H4" s="213"/>
       <c r="I4" s="213"/>
       <c r="J4" s="99"/>
       <c r="K4" s="213" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="L4" s="213"/>
       <c r="M4" s="213"/>
@@ -10034,7 +10039,7 @@
     </row>
     <row r="5" spans="1:14" ht="15.95" customHeight="1">
       <c r="A5" s="213" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B5" s="179"/>
       <c r="C5" s="179"/>
@@ -10300,21 +10305,21 @@
     </row>
     <row r="19" spans="1:14" ht="15.95" customHeight="1">
       <c r="A19" s="213" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B19" s="213"/>
       <c r="C19" s="213"/>
       <c r="D19" s="213"/>
       <c r="E19" s="99"/>
       <c r="F19" s="213" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="G19" s="213"/>
       <c r="H19" s="213"/>
       <c r="I19" s="213"/>
       <c r="J19" s="99"/>
       <c r="K19" s="213" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="L19" s="213"/>
       <c r="M19" s="213"/>
@@ -10327,7 +10332,7 @@
       <c r="D20" s="99"/>
       <c r="E20" s="99"/>
       <c r="F20" s="216" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="G20" s="216"/>
       <c r="H20" s="216"/>
@@ -10349,7 +10354,7 @@
       <c r="D21" s="214"/>
       <c r="E21" s="99"/>
       <c r="F21" s="216" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="G21" s="216"/>
       <c r="H21" s="216"/>
@@ -10391,7 +10396,7 @@
       <c r="D23" s="214"/>
       <c r="E23" s="99"/>
       <c r="F23" s="217" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="G23" s="217"/>
       <c r="H23" s="217"/>
@@ -10433,7 +10438,7 @@
       <c r="D25" s="214"/>
       <c r="E25" s="99"/>
       <c r="F25" s="133" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G25" s="133"/>
       <c r="H25" s="133"/>
@@ -10455,7 +10460,7 @@
       <c r="D26" s="214"/>
       <c r="E26" s="99"/>
       <c r="F26" s="133" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G26" s="133"/>
       <c r="H26" s="133"/>
@@ -10493,7 +10498,7 @@
       <c r="D28" s="214"/>
       <c r="E28" s="99"/>
       <c r="F28" s="133" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="G28" s="133"/>
       <c r="H28" s="133"/>
@@ -10513,7 +10518,7 @@
       <c r="D29" s="214"/>
       <c r="E29" s="99"/>
       <c r="F29" s="133" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="G29" s="133"/>
       <c r="H29" s="133"/>
@@ -10551,7 +10556,7 @@
       <c r="D31" s="214"/>
       <c r="E31" s="99"/>
       <c r="F31" s="133" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="G31" s="133"/>
       <c r="H31" s="133"/>
@@ -10571,7 +10576,7 @@
       <c r="D32" s="214"/>
       <c r="E32" s="99"/>
       <c r="F32" s="133" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="G32" s="133"/>
       <c r="H32" s="133"/>
@@ -10604,7 +10609,7 @@
       <c r="D34" s="214"/>
       <c r="E34" s="99"/>
       <c r="F34" s="133" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="G34" s="133"/>
       <c r="H34" s="133"/>
@@ -10619,7 +10624,7 @@
       <c r="D35" s="214"/>
       <c r="E35" s="99"/>
       <c r="F35" s="133" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="G35" s="133"/>
       <c r="H35" s="133"/>
@@ -10647,7 +10652,7 @@
       <c r="D37" s="214"/>
       <c r="E37" s="99"/>
       <c r="F37" s="133" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="G37" s="133"/>
       <c r="H37" s="133"/>
@@ -10675,7 +10680,7 @@
       <c r="D39" s="214"/>
       <c r="E39" s="99"/>
       <c r="F39" s="133" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="G39" s="133"/>
       <c r="H39" s="133"/>
@@ -10703,7 +10708,7 @@
       <c r="D41" s="214"/>
       <c r="E41" s="99"/>
       <c r="F41" s="217" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="G41" s="217"/>
       <c r="H41" s="217"/>
@@ -10959,7 +10964,7 @@
   <sheetData>
     <row r="2" spans="1:16" ht="21.75" customHeight="1">
       <c r="A2" s="139" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B2" s="181"/>
       <c r="C2" s="181"/>
@@ -10980,7 +10985,7 @@
     <row r="5" spans="1:16" ht="26.1" customHeight="1">
       <c r="A5" s="99"/>
       <c r="B5" s="224" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C5" s="221"/>
       <c r="D5" s="221"/>
@@ -11000,14 +11005,14 @@
     <row r="6" spans="1:16" ht="18" customHeight="1">
       <c r="A6" s="99"/>
       <c r="B6" s="218" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C6" s="179"/>
       <c r="D6" s="179" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E6" s="179" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F6" s="219"/>
       <c r="G6" s="179"/>
@@ -11015,7 +11020,7 @@
       <c r="I6" s="99"/>
       <c r="J6" s="99"/>
       <c r="K6" s="139" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="L6" s="139"/>
       <c r="M6" s="139"/>
@@ -11026,17 +11031,17 @@
     <row r="7" spans="1:16" ht="18" customHeight="1">
       <c r="A7" s="99"/>
       <c r="B7" s="136" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C7" s="115" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="D7" s="179"/>
       <c r="E7" s="115" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="F7" s="134" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="G7" s="115"/>
       <c r="H7" s="115"/>
@@ -11052,10 +11057,10 @@
     <row r="8" spans="1:16" ht="14.1" customHeight="1">
       <c r="A8" s="99"/>
       <c r="B8" s="136" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C8" s="115" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D8" s="115">
         <v>2</v>
@@ -11071,12 +11076,12 @@
       <c r="I8" s="99"/>
       <c r="J8" s="99"/>
       <c r="K8" s="220" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="L8" s="220"/>
       <c r="M8" s="220"/>
       <c r="N8" s="228" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="O8" s="228"/>
       <c r="P8" s="115"/>
@@ -11084,10 +11089,10 @@
     <row r="9" spans="1:16" ht="14.1" customHeight="1">
       <c r="A9" s="99"/>
       <c r="B9" s="136" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C9" s="115" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D9" s="115">
         <v>3</v>
@@ -11103,7 +11108,7 @@
       <c r="I9" s="99"/>
       <c r="J9" s="99"/>
       <c r="K9" s="220" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="L9" s="220"/>
       <c r="M9" s="220"/>
@@ -11116,10 +11121,10 @@
     <row r="10" spans="1:16" ht="14.1" customHeight="1">
       <c r="A10" s="99"/>
       <c r="B10" s="136" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C10" s="115" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D10" s="115">
         <v>5</v>
@@ -11135,12 +11140,12 @@
       <c r="I10" s="99"/>
       <c r="J10" s="99"/>
       <c r="K10" s="220" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="L10" s="220"/>
       <c r="M10" s="220"/>
       <c r="N10" s="228" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="O10" s="228"/>
       <c r="P10" s="115"/>
@@ -11148,10 +11153,10 @@
     <row r="11" spans="1:16" ht="14.1" customHeight="1">
       <c r="A11" s="99"/>
       <c r="B11" s="136" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C11" s="115" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D11" s="115">
         <v>9</v>
@@ -11167,7 +11172,7 @@
       <c r="I11" s="99"/>
       <c r="J11" s="99"/>
       <c r="K11" s="220" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="L11" s="220"/>
       <c r="M11" s="220"/>
@@ -11180,10 +11185,10 @@
     <row r="12" spans="1:16" ht="14.1" customHeight="1">
       <c r="A12" s="99"/>
       <c r="B12" s="136" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C12" s="115" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D12" s="115">
         <v>17</v>
@@ -11208,10 +11213,10 @@
     <row r="13" spans="1:16" ht="14.1" customHeight="1">
       <c r="A13" s="99"/>
       <c r="B13" s="136" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C13" s="115" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="D13" s="115">
         <v>33</v>
@@ -11236,10 +11241,10 @@
     <row r="14" spans="1:16" ht="14.1" customHeight="1">
       <c r="A14" s="99"/>
       <c r="B14" s="136" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C14" s="115" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D14" s="115">
         <v>65</v>
@@ -11264,10 +11269,10 @@
     <row r="15" spans="1:16" ht="14.1" customHeight="1">
       <c r="A15" s="99"/>
       <c r="B15" s="136" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C15" s="115" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D15" s="115">
         <v>129</v>
@@ -11292,10 +11297,10 @@
     <row r="16" spans="1:16" ht="14.1" customHeight="1">
       <c r="A16" s="99"/>
       <c r="B16" s="136" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C16" s="115" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D16" s="115">
         <v>257</v>
@@ -11319,10 +11324,10 @@
     </row>
     <row r="17" spans="2:16" ht="14.1" customHeight="1">
       <c r="B17" s="75" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C17" s="76" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D17" s="76">
         <v>513</v>
@@ -11346,7 +11351,7 @@
     </row>
     <row r="20" spans="2:16" ht="26.1" customHeight="1">
       <c r="B20" s="224" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C20" s="221"/>
       <c r="D20" s="221"/>
@@ -11365,21 +11370,21 @@
     </row>
     <row r="21" spans="2:16" ht="18" customHeight="1">
       <c r="B21" s="218" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C21" s="179"/>
       <c r="D21" s="179" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E21" s="179" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F21" s="219"/>
       <c r="G21" s="179"/>
       <c r="H21" s="179"/>
       <c r="I21" s="99"/>
       <c r="J21" s="139" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K21" s="179"/>
       <c r="L21" s="179"/>
@@ -11390,39 +11395,39 @@
     </row>
     <row r="22" spans="2:16" ht="18" customHeight="1">
       <c r="B22" s="136" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C22" s="115" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="D22" s="179"/>
       <c r="E22" s="115" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="F22" s="134" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="G22" s="115"/>
       <c r="H22" s="115"/>
       <c r="I22" s="99"/>
       <c r="J22" s="179" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K22" s="181"/>
       <c r="L22" s="181"/>
       <c r="M22" s="99"/>
       <c r="N22" s="179" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="O22" s="179"/>
       <c r="P22" s="181"/>
     </row>
     <row r="23" spans="2:16" ht="14.1" customHeight="1">
       <c r="B23" s="136" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C23" s="115" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D23" s="115">
         <v>1</v>
@@ -11437,23 +11442,23 @@
       <c r="H23" s="99"/>
       <c r="I23" s="99"/>
       <c r="J23" s="179" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K23" s="181"/>
       <c r="L23" s="181"/>
       <c r="M23" s="99"/>
       <c r="N23" s="179" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="O23" s="179"/>
       <c r="P23" s="181"/>
     </row>
     <row r="24" spans="2:16" ht="14.1" customHeight="1">
       <c r="B24" s="136" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="C24" s="115" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D24" s="115">
         <v>2</v>
@@ -11470,23 +11475,23 @@
       <c r="H24" s="99"/>
       <c r="I24" s="99"/>
       <c r="J24" s="179" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K24" s="181"/>
       <c r="L24" s="181"/>
       <c r="M24" s="99"/>
       <c r="N24" s="179" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="O24" s="179"/>
       <c r="P24" s="181"/>
     </row>
     <row r="25" spans="2:16" ht="14.1" customHeight="1">
       <c r="B25" s="136" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C25" s="115" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="D25" s="115">
         <v>4</v>
@@ -11502,7 +11507,7 @@
       <c r="H25" s="99"/>
       <c r="I25" s="99"/>
       <c r="J25" s="179" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="K25" s="179"/>
       <c r="L25" s="179"/>
@@ -11513,10 +11518,10 @@
     </row>
     <row r="26" spans="2:16" ht="14.1" customHeight="1">
       <c r="B26" s="136" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C26" s="115" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="D26" s="115">
         <v>8</v>
@@ -11541,10 +11546,10 @@
     </row>
     <row r="27" spans="2:16" ht="14.1" customHeight="1">
       <c r="B27" s="136" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C27" s="115" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D27" s="115">
         <v>16</v>
@@ -11569,10 +11574,10 @@
     </row>
     <row r="28" spans="2:16" ht="14.1" customHeight="1">
       <c r="B28" s="136" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C28" s="115" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="D28" s="115">
         <v>32</v>
@@ -11597,10 +11602,10 @@
     </row>
     <row r="29" spans="2:16" ht="14.1" customHeight="1">
       <c r="B29" s="136" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C29" s="115" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="D29" s="115">
         <v>64</v>
@@ -11625,10 +11630,10 @@
     </row>
     <row r="30" spans="2:16" ht="14.1" customHeight="1">
       <c r="B30" s="136" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C30" s="115" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="D30" s="115">
         <v>128</v>
@@ -11653,10 +11658,10 @@
     </row>
     <row r="31" spans="2:16" ht="14.1" customHeight="1">
       <c r="B31" s="75" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C31" s="76" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="D31" s="76">
         <v>256</v>
@@ -11706,7 +11711,7 @@
     </row>
     <row r="34" spans="2:8" ht="26.1" customHeight="1">
       <c r="B34" s="224" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C34" s="221"/>
       <c r="D34" s="221"/>
@@ -11717,14 +11722,14 @@
     </row>
     <row r="35" spans="2:8" ht="18" customHeight="1">
       <c r="B35" s="218" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C35" s="179"/>
       <c r="D35" s="179" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E35" s="179" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F35" s="219"/>
       <c r="G35" s="179"/>
@@ -11732,22 +11737,22 @@
     </row>
     <row r="36" spans="2:8" ht="18" customHeight="1">
       <c r="B36" s="136" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="C36" s="115"/>
       <c r="D36" s="179"/>
       <c r="E36" s="115" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="F36" s="134" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="G36" s="115"/>
       <c r="H36" s="115"/>
     </row>
     <row r="37" spans="2:8" ht="14.1" customHeight="1">
       <c r="B37" s="136" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C37" s="115"/>
       <c r="D37" s="115">
@@ -11762,7 +11767,7 @@
     </row>
     <row r="38" spans="2:8" ht="14.1" customHeight="1">
       <c r="B38" s="136" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="C38" s="115"/>
       <c r="D38" s="115">
@@ -11778,7 +11783,7 @@
     </row>
     <row r="39" spans="2:8" ht="14.1" customHeight="1">
       <c r="B39" s="136" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C39" s="115"/>
       <c r="D39" s="115">
@@ -11793,7 +11798,7 @@
     </row>
     <row r="40" spans="2:8" ht="14.1" customHeight="1">
       <c r="B40" s="136" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C40" s="115"/>
       <c r="D40" s="115">
@@ -11808,7 +11813,7 @@
     </row>
     <row r="41" spans="2:8" ht="14.1" customHeight="1">
       <c r="B41" s="136" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C41" s="115"/>
       <c r="D41" s="115">
@@ -11823,7 +11828,7 @@
     </row>
     <row r="42" spans="2:8" ht="14.1" customHeight="1">
       <c r="B42" s="136" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C42" s="115"/>
       <c r="D42" s="115">
@@ -11838,7 +11843,7 @@
     </row>
     <row r="43" spans="2:8" ht="14.1" customHeight="1">
       <c r="B43" s="136" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C43" s="115"/>
       <c r="D43" s="115">
@@ -11853,7 +11858,7 @@
     </row>
     <row r="44" spans="2:8" ht="14.1" customHeight="1">
       <c r="B44" s="136" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C44" s="115"/>
       <c r="D44" s="115">
@@ -11868,7 +11873,7 @@
     </row>
     <row r="45" spans="2:8" ht="14.1" customHeight="1">
       <c r="B45" s="75" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C45" s="76"/>
       <c r="D45" s="76">
@@ -11883,7 +11888,7 @@
     </row>
     <row r="48" spans="2:8" ht="26.1" customHeight="1">
       <c r="B48" s="221" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C48" s="221"/>
       <c r="D48" s="221"/>
@@ -11894,14 +11899,14 @@
     </row>
     <row r="49" spans="2:8" ht="18" customHeight="1">
       <c r="B49" s="179" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C49" s="179"/>
       <c r="D49" s="179" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E49" s="179" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F49" s="219"/>
       <c r="G49" s="179"/>
@@ -11912,17 +11917,17 @@
       <c r="C50" s="99"/>
       <c r="D50" s="179"/>
       <c r="E50" s="115" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="F50" s="134" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="G50" s="115"/>
       <c r="H50" s="115"/>
     </row>
     <row r="51" spans="2:8" ht="14.1" customHeight="1">
       <c r="B51" s="115" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C51" s="99"/>
       <c r="D51" s="115">
@@ -11939,7 +11944,7 @@
     </row>
     <row r="52" spans="2:8" ht="14.1" customHeight="1">
       <c r="B52" s="115" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="C52" s="99"/>
       <c r="D52" s="115">
@@ -11956,7 +11961,7 @@
     </row>
     <row r="53" spans="2:8" ht="14.1" customHeight="1">
       <c r="B53" s="115" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C53" s="99"/>
       <c r="D53" s="115">
@@ -11973,7 +11978,7 @@
     </row>
     <row r="54" spans="2:8" ht="14.1" customHeight="1">
       <c r="B54" s="107" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="C54" s="79"/>
       <c r="D54" s="107">
@@ -11990,7 +11995,7 @@
     </row>
     <row r="55" spans="2:8" ht="14.1" customHeight="1">
       <c r="B55" s="115" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C55" s="99"/>
       <c r="D55" s="115">
@@ -12007,7 +12012,7 @@
     </row>
     <row r="56" spans="2:8" ht="14.1" customHeight="1">
       <c r="B56" s="107" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C56" s="79"/>
       <c r="D56" s="107">
@@ -12024,7 +12029,7 @@
     </row>
     <row r="57" spans="2:8" ht="14.1" customHeight="1">
       <c r="B57" s="107" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C57" s="79"/>
       <c r="D57" s="107">
@@ -12041,7 +12046,7 @@
     </row>
     <row r="58" spans="2:8" ht="14.1" customHeight="1">
       <c r="B58" s="107" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="C58" s="79"/>
       <c r="D58" s="107">
@@ -12058,7 +12063,7 @@
     </row>
     <row r="59" spans="2:8" ht="14.1" customHeight="1">
       <c r="B59" s="115" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C59" s="99"/>
       <c r="D59" s="115">
@@ -12075,7 +12080,7 @@
     </row>
     <row r="60" spans="2:8" ht="14.1" customHeight="1">
       <c r="B60" s="107" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="C60" s="79"/>
       <c r="D60" s="107">
@@ -12092,7 +12097,7 @@
     </row>
     <row r="61" spans="2:8" ht="14.1" customHeight="1">
       <c r="B61" s="115" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C61" s="99"/>
       <c r="D61" s="119">
@@ -12109,7 +12114,7 @@
     </row>
     <row r="62" spans="2:8" ht="14.1" customHeight="1">
       <c r="B62" s="107" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="C62" s="79"/>
       <c r="D62" s="107">
@@ -12126,7 +12131,7 @@
     </row>
     <row r="63" spans="2:8" ht="14.1" customHeight="1">
       <c r="B63" s="76" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C63" s="80"/>
       <c r="D63" s="76">
@@ -12143,7 +12148,7 @@
     </row>
     <row r="64" spans="2:8" ht="14.1" customHeight="1">
       <c r="B64" s="223" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="C64" s="223"/>
       <c r="D64" s="223"/>
@@ -12154,7 +12159,7 @@
     </row>
     <row r="67" spans="2:8" ht="26.1" customHeight="1">
       <c r="B67" s="224" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="C67" s="221"/>
       <c r="D67" s="221"/>
@@ -12165,14 +12170,14 @@
     </row>
     <row r="68" spans="2:8" ht="18" customHeight="1">
       <c r="B68" s="218" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C68" s="179"/>
       <c r="D68" s="179" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E68" s="179" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F68" s="219"/>
       <c r="G68" s="179"/>
@@ -12180,22 +12185,22 @@
     </row>
     <row r="69" spans="2:8" ht="18" customHeight="1">
       <c r="B69" s="136" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="C69" s="99"/>
       <c r="D69" s="179"/>
       <c r="E69" s="115" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="F69" s="134" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="G69" s="115"/>
       <c r="H69" s="115"/>
     </row>
     <row r="70" spans="2:8" ht="14.1" customHeight="1">
       <c r="B70" s="136" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C70" s="99"/>
       <c r="D70" s="115">
@@ -12212,7 +12217,7 @@
     </row>
     <row r="71" spans="2:8" ht="14.1" customHeight="1">
       <c r="B71" s="136" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="C71" s="99"/>
       <c r="D71" s="115">
@@ -12229,7 +12234,7 @@
     </row>
     <row r="72" spans="2:8" ht="14.1" customHeight="1">
       <c r="B72" s="136" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C72" s="99"/>
       <c r="D72" s="115">
@@ -12246,7 +12251,7 @@
     </row>
     <row r="73" spans="2:8" ht="14.1" customHeight="1">
       <c r="B73" s="110" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="C73" s="111"/>
       <c r="D73" s="107">
@@ -12263,7 +12268,7 @@
     </row>
     <row r="74" spans="2:8" ht="14.1" customHeight="1">
       <c r="B74" s="136" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C74" s="99"/>
       <c r="D74" s="115">
@@ -12280,7 +12285,7 @@
     </row>
     <row r="75" spans="2:8" ht="14.1" customHeight="1">
       <c r="B75" s="110" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="C75" s="111"/>
       <c r="D75" s="107">
@@ -12297,7 +12302,7 @@
     </row>
     <row r="76" spans="2:8" ht="14.1" customHeight="1">
       <c r="B76" s="136" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="C76" s="99"/>
       <c r="D76" s="115">
@@ -12314,7 +12319,7 @@
     </row>
     <row r="77" spans="2:8" ht="14.1" customHeight="1">
       <c r="B77" s="110" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="C77" s="111"/>
       <c r="D77" s="107">
@@ -12331,7 +12336,7 @@
     </row>
     <row r="78" spans="2:8" ht="14.1" customHeight="1">
       <c r="B78" s="136" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="C78" s="99"/>
       <c r="D78" s="115">
@@ -12348,7 +12353,7 @@
     </row>
     <row r="79" spans="2:8" ht="14.1" customHeight="1">
       <c r="B79" s="110" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="C79" s="111"/>
       <c r="D79" s="107">
@@ -12365,7 +12370,7 @@
     </row>
     <row r="80" spans="2:8" ht="14.1" customHeight="1">
       <c r="B80" s="136" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="C80" s="99"/>
       <c r="D80" s="115">
@@ -12382,7 +12387,7 @@
     </row>
     <row r="81" spans="2:8" ht="14.1" customHeight="1">
       <c r="B81" s="110" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C81" s="111"/>
       <c r="D81" s="107">
@@ -12399,7 +12404,7 @@
     </row>
     <row r="82" spans="2:8" ht="14.1" customHeight="1">
       <c r="B82" s="75" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C82" s="80"/>
       <c r="D82" s="76">
@@ -12416,7 +12421,7 @@
     </row>
     <row r="83" spans="2:8" ht="14.1" customHeight="1">
       <c r="B83" s="223" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="C83" s="223"/>
       <c r="D83" s="223"/>
@@ -12427,7 +12432,7 @@
     </row>
     <row r="86" spans="2:8" ht="26.1" customHeight="1">
       <c r="B86" s="225" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="C86" s="226"/>
       <c r="D86" s="226"/>
@@ -12438,14 +12443,14 @@
     </row>
     <row r="87" spans="2:8" ht="18" customHeight="1">
       <c r="B87" s="218" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C87" s="179"/>
       <c r="D87" s="179" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E87" s="179" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F87" s="219"/>
       <c r="G87" s="179"/>
@@ -12456,17 +12461,17 @@
       <c r="C88" s="99"/>
       <c r="D88" s="179"/>
       <c r="E88" s="115" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="F88" s="134" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="G88" s="115"/>
       <c r="H88" s="115"/>
     </row>
     <row r="89" spans="2:8" ht="14.1" customHeight="1">
       <c r="B89" s="136" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C89" s="115"/>
       <c r="D89" s="115">
@@ -12481,7 +12486,7 @@
     </row>
     <row r="90" spans="2:8" ht="14.1" customHeight="1">
       <c r="B90" s="136" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="C90" s="115"/>
       <c r="D90" s="115">
@@ -12496,7 +12501,7 @@
     </row>
     <row r="91" spans="2:8" ht="14.1" customHeight="1">
       <c r="B91" s="136" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C91" s="115"/>
       <c r="D91" s="115">
@@ -12511,7 +12516,7 @@
     </row>
     <row r="92" spans="2:8" ht="14.1" customHeight="1">
       <c r="B92" s="136" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="C92" s="115"/>
       <c r="D92" s="115">
@@ -12526,7 +12531,7 @@
     </row>
     <row r="93" spans="2:8" ht="14.1" customHeight="1">
       <c r="B93" s="136" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C93" s="115"/>
       <c r="D93" s="115">
@@ -12541,7 +12546,7 @@
     </row>
     <row r="94" spans="2:8" ht="14.1" customHeight="1">
       <c r="B94" s="136" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C94" s="115"/>
       <c r="D94" s="115">
@@ -12556,7 +12561,7 @@
     </row>
     <row r="95" spans="2:8" ht="14.1" customHeight="1">
       <c r="B95" s="136" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C95" s="115"/>
       <c r="D95" s="115">
@@ -12571,7 +12576,7 @@
     </row>
     <row r="96" spans="2:8" ht="14.1" customHeight="1">
       <c r="B96" s="136" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C96" s="115"/>
       <c r="D96" s="115">
@@ -12586,7 +12591,7 @@
     </row>
     <row r="97" spans="2:6" ht="14.1" customHeight="1">
       <c r="B97" s="136" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C97" s="115"/>
       <c r="D97" s="115">
@@ -12599,7 +12604,7 @@
     </row>
     <row r="98" spans="2:6" ht="14.1" customHeight="1">
       <c r="B98" s="136" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="C98" s="115"/>
       <c r="D98" s="115">
@@ -12612,7 +12617,7 @@
     </row>
     <row r="99" spans="2:6" ht="14.1" customHeight="1">
       <c r="B99" s="136" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C99" s="115"/>
       <c r="D99" s="115">
@@ -12625,7 +12630,7 @@
     </row>
     <row r="100" spans="2:6" ht="14.1" customHeight="1">
       <c r="B100" s="136" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C100" s="115"/>
       <c r="D100" s="115">
@@ -12638,7 +12643,7 @@
     </row>
     <row r="101" spans="2:6" ht="14.1" customHeight="1">
       <c r="B101" s="136" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C101" s="115"/>
       <c r="D101" s="115">
@@ -12651,7 +12656,7 @@
     </row>
     <row r="102" spans="2:6" ht="14.1" customHeight="1">
       <c r="B102" s="136" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C102" s="115"/>
       <c r="D102" s="115">
@@ -12664,7 +12669,7 @@
     </row>
     <row r="103" spans="2:6" ht="14.1" customHeight="1">
       <c r="B103" s="75" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="C103" s="76"/>
       <c r="D103" s="76">

</xml_diff>